<commit_message>
corrected the inconsistent codes in the manual coding.
</commit_message>
<xml_diff>
--- a/data/comments/comments_manual_coding.xlsx
+++ b/data/comments/comments_manual_coding.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joellattmann/Documents/GitHub/like_dislike/data/comments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yuginkha/Documents/Mediapsychology/like_dislike/data/comments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C29023-2BF9-4546-A641-338CE6211489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D6CD28-95C9-634C-BA36-DBFBB33F6CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{C1BB1A16-32F0-7443-88B2-C6116B7B62A9}"/>
   </bookViews>
@@ -1632,7 +1632,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1640,18 +1640,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1671,7 +1681,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2100,7 +2110,7 @@
         <v>1</v>
       </c>
       <c r="I2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J2">
         <v>3</v>
@@ -2268,7 +2278,7 @@
         <v>1</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J6">
         <v>3</v>
@@ -2346,19 +2356,19 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="s">
         <v>42</v>
@@ -2397,13 +2407,13 @@
         <v>1</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9">
         <v>2</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" t="s">
         <v>47</v>
@@ -2442,7 +2452,7 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -2475,10 +2485,10 @@
         <v>52</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -2487,10 +2497,10 @@
         <v>1</v>
       </c>
       <c r="J11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="s">
         <v>53</v>
@@ -2577,10 +2587,10 @@
         <v>2</v>
       </c>
       <c r="J13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" t="s">
         <v>61</v>
@@ -2610,19 +2620,19 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
         <v>1</v>
       </c>
       <c r="J14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="s">
         <v>64</v>
@@ -2658,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15">
         <v>3</v>
@@ -2703,7 +2713,7 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16">
         <v>3</v>
@@ -2748,10 +2758,10 @@
         <v>1</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="s">
         <v>75</v>
@@ -2787,10 +2797,10 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -2832,7 +2842,7 @@
         <v>1</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19">
         <v>3</v>
@@ -2874,7 +2884,7 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20">
         <v>4</v>
@@ -2892,7 +2902,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2909,22 +2919,22 @@
       <c r="E21" t="s">
         <v>87</v>
       </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="H21">
-        <v>0</v>
-      </c>
-      <c r="I21">
-        <v>0</v>
-      </c>
-      <c r="J21">
-        <v>1</v>
-      </c>
-      <c r="K21">
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2">
+        <v>3</v>
+      </c>
+      <c r="K21" s="2">
         <v>0</v>
       </c>
       <c r="L21" t="s">
@@ -3197,7 +3207,7 @@
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28">
-        <f t="shared" si="0"/>
+        <f>ROW()-1</f>
         <v>27</v>
       </c>
       <c r="B28">
@@ -3219,7 +3229,7 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28">
         <v>2</v>
@@ -4119,7 +4129,7 @@
         <v>1</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49">
         <v>2</v>
@@ -4533,7 +4543,7 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H58">
         <v>0</v>
@@ -4635,7 +4645,7 @@
         <v>1</v>
       </c>
       <c r="I60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60">
         <v>2</v>
@@ -4929,7 +4939,7 @@
         <v>0</v>
       </c>
       <c r="H66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66">
         <v>2</v>
@@ -5082,7 +5092,7 @@
         <v>2</v>
       </c>
       <c r="K69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" t="s">
         <v>246</v>
@@ -5118,7 +5128,7 @@
         <v>0</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -5130,7 +5140,7 @@
         <v>2</v>
       </c>
       <c r="K70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L70" t="s">
         <v>249</v>
@@ -5271,7 +5281,7 @@
         <v>0</v>
       </c>
       <c r="I73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J73">
         <v>2</v>
@@ -5319,7 +5329,7 @@
         <v>1</v>
       </c>
       <c r="I74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J74">
         <v>3</v>
@@ -5520,7 +5530,7 @@
         <v>2</v>
       </c>
       <c r="K78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L78" t="s">
         <v>272</v>
@@ -5616,10 +5626,10 @@
         <v>2</v>
       </c>
       <c r="J80">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L80" t="s">
         <v>278</v>
@@ -6240,7 +6250,7 @@
         <v>0</v>
       </c>
       <c r="I93">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J93">
         <v>2</v>
@@ -6576,13 +6586,13 @@
         <v>0</v>
       </c>
       <c r="H100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I100">
         <v>2</v>
       </c>
       <c r="J100">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K100">
         <v>0</v>
@@ -6627,7 +6637,7 @@
         <v>0</v>
       </c>
       <c r="I101">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J101">
         <v>4</v>
@@ -6936,7 +6946,7 @@
         <v>365</v>
       </c>
       <c r="F107">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G107">
         <v>0</v>
@@ -6948,7 +6958,7 @@
         <v>4</v>
       </c>
       <c r="J107">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K107">
         <v>0</v>
@@ -7212,7 +7222,7 @@
         <v>0</v>
       </c>
       <c r="H112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112">
         <v>1</v>
@@ -7266,7 +7276,7 @@
         <v>0</v>
       </c>
       <c r="G113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H113">
         <v>0</v>
@@ -7329,7 +7339,7 @@
         <v>0</v>
       </c>
       <c r="I114">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J114">
         <v>1</v>
@@ -7812,16 +7822,16 @@
         <v>0</v>
       </c>
       <c r="H123">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I123">
         <v>2</v>
       </c>
       <c r="J123">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K123">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L123" t="s">
         <v>424</v>
@@ -8034,7 +8044,7 @@
         <v>0</v>
       </c>
       <c r="I127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J127">
         <v>3</v>
@@ -8088,7 +8098,7 @@
         <v>0</v>
       </c>
       <c r="I128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128">
         <v>1</v>
@@ -8463,13 +8473,13 @@
         <v>0</v>
       </c>
       <c r="G135">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H135">
         <v>1</v>
       </c>
       <c r="I135">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J135">
         <v>2</v>
@@ -8634,7 +8644,7 @@
         <v>0</v>
       </c>
       <c r="J138">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K138">
         <v>0</v>
@@ -9009,7 +9019,7 @@
         <v>1</v>
       </c>
       <c r="H145">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I145">
         <v>2</v>
@@ -9234,7 +9244,7 @@
         <v>0</v>
       </c>
       <c r="J149">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K149">
         <v>0</v>
@@ -9342,7 +9352,7 @@
         <v>0</v>
       </c>
       <c r="J151">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K151">
         <v>0</v>

</xml_diff>